<commit_message>
Add ACI learning-rate modulation with spectral capping and Mondrian per-regime coverage tracking
</commit_message>
<xml_diff>
--- a/results/adaptive_conformal_results.xlsx
+++ b/results/adaptive_conformal_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
   <si>
     <t>setting</t>
   </si>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -488,6 +488,58 @@
         <v>0.0633851560339848</v>
       </c>
     </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>0.9</v>
+      </c>
+      <c r="D4">
+        <v>0.71</v>
+      </c>
+      <c r="E4">
+        <v>0.0051882933974932</v>
+      </c>
+      <c r="F4">
+        <v>0.1206913095790929</v>
+      </c>
+      <c r="G4">
+        <v>0.0013346303412346</v>
+      </c>
+      <c r="H4">
+        <v>0.0477916956805662</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>0.9</v>
+      </c>
+      <c r="D5">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="E5">
+        <v>0.007927865059397</v>
+      </c>
+      <c r="F5">
+        <v>0.08901465169859291</v>
+      </c>
+      <c r="G5">
+        <v>0.0029202803524616</v>
+      </c>
+      <c r="H5">
+        <v>0.0402981693713987</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add CQR-inspired single-score conformal correction with empirical base quantiles and finite-sample coverage guarantee
</commit_message>
<xml_diff>
--- a/results/adaptive_conformal_results.xlsx
+++ b/results/adaptive_conformal_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
   <si>
     <t>setting</t>
   </si>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -540,6 +540,32 @@
         <v>0.0402981693713987</v>
       </c>
     </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>0.9</v>
+      </c>
+      <c r="D6">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="E6">
+        <v>0.0045473414355612</v>
+      </c>
+      <c r="F6">
+        <v>0.0815688521412361</v>
+      </c>
+      <c r="G6">
+        <v>0.0033975786240265</v>
+      </c>
+      <c r="H6">
+        <v>0.0677489747453449</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace empirical base quantiles with online CQR using periodic quantile regression on calibration buffer with sequential split for finite-sample validity
</commit_message>
<xml_diff>
--- a/results/adaptive_conformal_results.xlsx
+++ b/results/adaptive_conformal_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
   <si>
     <t>setting</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t>conformal_acp_lags96_modellinear_cpacp_a0.1_cw200_seed0_modeonline_debug-0_M0</t>
+  </si>
+  <si>
+    <t>exchange_rate.csv_lags96_modellinear_cpacp_modeonline_seed0</t>
   </si>
   <si>
     <t>acp</t>
@@ -404,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -441,7 +444,7 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>0.9</v>
@@ -467,7 +470,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>0.9</v>
@@ -493,7 +496,7 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>0.9</v>
@@ -519,7 +522,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>0.9</v>
@@ -545,7 +548,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>0.9</v>
@@ -564,6 +567,32 @@
       </c>
       <c r="H6">
         <v>0.0677489747453449</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>0.9</v>
+      </c>
+      <c r="D7">
+        <v>0.86</v>
+      </c>
+      <c r="E7">
+        <v>0.0024618431769066</v>
+      </c>
+      <c r="F7">
+        <v>0.0412860371103684</v>
+      </c>
+      <c r="G7">
+        <v>0.0018761254375603</v>
+      </c>
+      <c r="H7">
+        <v>0.0443215147859572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>